<commit_message>
feat(salud): MITs con backlog real en Tareas, sin desaparecer solos
Rediseno pedido tras probar el cierre: los MITs no resueltos ya NO se
pierden al dia siguiente. Ahora:
- registrar_mits crea filas en Tareas (Tipo=MIT, Fecha objetivo=manana)
  en vez de escribir texto libre en Diario. Reusa la hoja Tareas que
  ya existia (Estado/Completada) en vez de inventar un backlog propio.
- mits_pendientes() lee TODOS los MIT sin completar (hoy + acumulados,
  sin limite) para el panel del cierre; cada uno se marca por separado
  y tocar de nuevo lo desmarca (marcar_mit).
- senal_mits_brief() separa "de hoy" (Fecha objetivo=hoy) de
  "acumulados" (de antes) en el brief de las 8:00 -- solo informa, no
  pide nada (el brief sigue siendo de solo lectura).

Se retiran del schema hacia adelante las columnas Diario "MITs de
manana"/"MITs cumplidos" (quedan vacias en la planilla real como
artefacto sin uso, no se borran). 20 evals nuevos/reescritos.
</commit_message>
<xml_diff>
--- a/docs/Donna_Canonico.xlsx
+++ b/docs/Donna_Canonico.xlsx
@@ -2531,27 +2531,27 @@
           <t>Notas</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="35" t="inlineStr">
         <is>
           <t>Primera comida</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N2" s="35" t="inlineStr">
         <is>
           <t>Hora desperté</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O2" s="35" t="inlineStr">
         <is>
           <t>Agua</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" s="35" t="inlineStr">
         <is>
           <t>Proteína</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="35" t="inlineStr">
         <is>
           <t>Peso (kg)</t>
         </is>
@@ -3459,22 +3459,22 @@
           <t>👶 Tiempo hijo</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="35" t="inlineStr">
         <is>
           <t>Score hábitos</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" s="35" t="inlineStr">
         <is>
           <t>Ventana comida</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" s="35" t="inlineStr">
         <is>
           <t>Ventana sueño</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U2" s="35" t="inlineStr">
         <is>
           <t>Peso</t>
         </is>

</xml_diff>